<commit_message>
rec no R_a no Conj
</commit_message>
<xml_diff>
--- a/Experiment 1/Time_for_Bac_Fix_All_Subjects.xlsx
+++ b/Experiment 1/Time_for_Bac_Fix_All_Subjects.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\Experiment 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A564357C-311C-4132-98CE-7AD86745A6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4120B73E-7ED2-4DB8-B1E7-CA244F808A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{74D36821-7AB3-48D6-B8A7-7A9E8E7BAA96}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{74D36821-7AB3-48D6-B8A7-7A9E8E7BAA96}"/>
   </bookViews>
   <sheets>
     <sheet name="All Time Distributions" sheetId="3" r:id="rId1"/>
     <sheet name="Normal Equation" sheetId="1" r:id="rId2"/>
-    <sheet name="No R_a with Conjugation" sheetId="2" r:id="rId3"/>
+    <sheet name="No R_a with Conj" sheetId="2" r:id="rId3"/>
+    <sheet name="No R_a No Conj" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="5">
   <si>
     <t>Time_s</t>
   </si>
@@ -1070,4 +1071,160 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90EE3171-995E-4B1B-8577-D5D61727A24E}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>24167</v>
+      </c>
+      <c r="B2">
+        <f>A2/60</f>
+        <v>402.78333333333336</v>
+      </c>
+      <c r="C2">
+        <f>A2/3600</f>
+        <v>6.713055555555556</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>20031</v>
+      </c>
+      <c r="B3">
+        <f t="shared" ref="B3:B11" si="0">A3/60</f>
+        <v>333.85</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C11" si="1">A3/3600</f>
+        <v>5.5641666666666669</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>17489</v>
+      </c>
+      <c r="B4">
+        <f t="shared" si="0"/>
+        <v>291.48333333333335</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="1"/>
+        <v>4.8580555555555556</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>21330</v>
+      </c>
+      <c r="B5">
+        <f t="shared" si="0"/>
+        <v>355.5</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="1"/>
+        <v>5.9249999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>19687</v>
+      </c>
+      <c r="B6">
+        <f t="shared" si="0"/>
+        <v>328.11666666666667</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="1"/>
+        <v>5.4686111111111115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>20152</v>
+      </c>
+      <c r="B7">
+        <f t="shared" si="0"/>
+        <v>335.86666666666667</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="1"/>
+        <v>5.597777777777778</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>22159</v>
+      </c>
+      <c r="B8">
+        <f t="shared" si="0"/>
+        <v>369.31666666666666</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="1"/>
+        <v>6.1552777777777781</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>20647</v>
+      </c>
+      <c r="B9">
+        <f t="shared" si="0"/>
+        <v>344.11666666666667</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="1"/>
+        <v>5.7352777777777781</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>18862</v>
+      </c>
+      <c r="B10">
+        <f t="shared" si="0"/>
+        <v>314.36666666666667</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="1"/>
+        <v>5.2394444444444446</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>21400</v>
+      </c>
+      <c r="B11">
+        <f t="shared" si="0"/>
+        <v>356.66666666666669</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="1"/>
+        <v>5.9444444444444446</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added more data, plotting, and analysis
</commit_message>
<xml_diff>
--- a/Experiment 1/Time_for_Bac_Fix_All_Subjects.xlsx
+++ b/Experiment 1/Time_for_Bac_Fix_All_Subjects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\Experiment 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A050F307-A154-4AE2-A6D1-208C6A44D8E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4187566A-558F-4A1F-876B-F7C307E0D55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{74D36821-7AB3-48D6-B8A7-7A9E8E7BAA96}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="18675" windowHeight="12975" activeTab="3" xr2:uid="{74D36821-7AB3-48D6-B8A7-7A9E8E7BAA96}"/>
   </bookViews>
   <sheets>
     <sheet name="All Time Distributions" sheetId="3" r:id="rId1"/>
@@ -542,6 +542,9 @@
       <c r="B12">
         <v>18213</v>
       </c>
+      <c r="C12">
+        <v>15281</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -550,6 +553,9 @@
       <c r="B13">
         <v>17994</v>
       </c>
+      <c r="C13">
+        <v>20943</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -558,6 +564,9 @@
       <c r="B14">
         <v>22789</v>
       </c>
+      <c r="C14">
+        <v>20142</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -566,6 +575,9 @@
       <c r="B15">
         <v>20652</v>
       </c>
+      <c r="C15">
+        <v>17416</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -574,45 +586,63 @@
       <c r="B16">
         <v>14313</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <v>17469</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>18412</v>
       </c>
       <c r="B17">
         <v>18242</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>22998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>23735</v>
       </c>
       <c r="B18">
         <v>19832</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <v>19695</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18310</v>
       </c>
       <c r="B19">
         <v>21581</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <v>24320</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16977</v>
       </c>
       <c r="B20">
         <v>16294</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <v>24251</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20946</v>
       </c>
       <c r="B21">
         <v>17948</v>
+      </c>
+      <c r="C21">
+        <v>17664</v>
       </c>
     </row>
   </sheetData>
@@ -1112,7 +1142,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90EE3171-995E-4B1B-8577-D5D61727A24E}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -1261,6 +1291,118 @@
         <v>5.9444444444444446</v>
       </c>
     </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>15281</v>
+      </c>
+      <c r="B12">
+        <v>254.68333333333334</v>
+      </c>
+      <c r="C12">
+        <v>4.2447222222222223</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>20943</v>
+      </c>
+      <c r="B13">
+        <v>349.05</v>
+      </c>
+      <c r="C13">
+        <v>5.8174999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>20142</v>
+      </c>
+      <c r="B14">
+        <v>335.7</v>
+      </c>
+      <c r="C14">
+        <v>5.5949999999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>17416</v>
+      </c>
+      <c r="B15">
+        <v>290.26666666666665</v>
+      </c>
+      <c r="C15">
+        <v>4.8377777777777782</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>17469</v>
+      </c>
+      <c r="B16">
+        <v>291.14999999999998</v>
+      </c>
+      <c r="C16">
+        <v>4.8525</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>22998</v>
+      </c>
+      <c r="B17">
+        <v>383.3</v>
+      </c>
+      <c r="C17">
+        <v>6.3883333333333336</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>19695</v>
+      </c>
+      <c r="B18">
+        <f>A18/60</f>
+        <v>328.25</v>
+      </c>
+      <c r="C18">
+        <f>A18/3600</f>
+        <v>5.4708333333333332</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>24320</v>
+      </c>
+      <c r="B19">
+        <v>405.33333333333331</v>
+      </c>
+      <c r="C19">
+        <v>6.7555555555555555</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>24251</v>
+      </c>
+      <c r="B20">
+        <v>404.18333333333334</v>
+      </c>
+      <c r="C20">
+        <v>6.7363888888888885</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>17664</v>
+      </c>
+      <c r="B21">
+        <v>294.39999999999998</v>
+      </c>
+      <c r="C21">
+        <v>4.9066666666666663</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>